<commit_message>
updating suisun data again
</commit_message>
<xml_diff>
--- a/data-raw/Suisun/Suisun comments.xlsx
+++ b/data-raw/Suisun/Suisun comments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sbashevkin\Documents\LTMRdata\data-raw\Suisun\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD895961-1226-4B88-9051-1B38596C0823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E20A18AE-E83B-43E5-8B6D-6816A0CD43B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10339" uniqueCount="3747">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10363" uniqueCount="3765">
   <si>
     <t>SampleRowID</t>
   </si>
@@ -11272,6 +11272,60 @@
   </si>
   <si>
     <t>age-1 fish</t>
+  </si>
+  <si>
+    <t>{7A4D29B0-FDDB-42FA-87AF-1E090C87BA6A}</t>
+  </si>
+  <si>
+    <t>2026-01-23T08:00:00Z</t>
+  </si>
+  <si>
+    <t>2026-01-23T23:14:00Z</t>
+  </si>
+  <si>
+    <t>Suisun {7A4D29B0-FDDB-42FA-87AF-1E090C87BA6A}</t>
+  </si>
+  <si>
+    <t>Rhithropanopeus harrisii</t>
+  </si>
+  <si>
+    <t>Only caught one HARRISMC, this one is not a catch</t>
+  </si>
+  <si>
+    <t>{2EEC81E3-D5AE-40E1-B205-707C05C0417A}</t>
+  </si>
+  <si>
+    <t>2025-06-11T07:00:00Z</t>
+  </si>
+  <si>
+    <t>2025-06-11T14:54:00Z</t>
+  </si>
+  <si>
+    <t>Suisun {2EEC81E3-D5AE-40E1-B205-707C05C0417A}</t>
+  </si>
+  <si>
+    <t>Gammaridea</t>
+  </si>
+  <si>
+    <t>Not in count - DB won't delete</t>
+  </si>
+  <si>
+    <t>{E9C1D433-16E8-47A1-ABAF-07A1C5A8B24B}</t>
+  </si>
+  <si>
+    <t>2025-12-10T08:00:00Z</t>
+  </si>
+  <si>
+    <t>2025-12-10T18:11:00Z</t>
+  </si>
+  <si>
+    <t>Suisun {E9C1D433-16E8-47A1-ABAF-07A1C5A8B24B}</t>
+  </si>
+  <si>
+    <t>New hazard in the water -- started more downstream</t>
+  </si>
+  <si>
+    <t>Accidentally added extra row-- zero intentional</t>
   </si>
 </sst>
 </file>
@@ -12146,7 +12200,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O1258"/>
+  <dimension ref="A1:O1261"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.7109375" bestFit="1" customWidth="1"/>
@@ -53196,6 +53250,114 @@
       </c>
       <c r="N1258"/>
     </row>
+    <row r="1259" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1259" t="s">
+        <v>3747</v>
+      </c>
+      <c r="B1259" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1259" t="s">
+        <v>3748</v>
+      </c>
+      <c r="D1259" t="s">
+        <v>3749</v>
+      </c>
+      <c r="E1259" t="s">
+        <v>3750</v>
+      </c>
+      <c r="F1259" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1259" t="s">
+        <v>3751</v>
+      </c>
+      <c r="H1259">
+        <v>2</v>
+      </c>
+      <c r="I1259" t="s">
+        <v>3752</v>
+      </c>
+      <c r="J1259"/>
+      <c r="K1259"/>
+      <c r="L1259"/>
+      <c r="M1259"/>
+      <c r="N1259">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1260" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1260" t="s">
+        <v>3753</v>
+      </c>
+      <c r="B1260" t="s">
+        <v>213</v>
+      </c>
+      <c r="C1260" t="s">
+        <v>3754</v>
+      </c>
+      <c r="D1260" t="s">
+        <v>3755</v>
+      </c>
+      <c r="E1260" t="s">
+        <v>3756</v>
+      </c>
+      <c r="F1260" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1260" t="s">
+        <v>3757</v>
+      </c>
+      <c r="H1260">
+        <v>2</v>
+      </c>
+      <c r="I1260" t="s">
+        <v>3758</v>
+      </c>
+      <c r="J1260"/>
+      <c r="K1260"/>
+      <c r="L1260"/>
+      <c r="M1260"/>
+      <c r="N1260">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1261" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1261" t="s">
+        <v>3759</v>
+      </c>
+      <c r="B1261" t="s">
+        <v>213</v>
+      </c>
+      <c r="C1261" t="s">
+        <v>3760</v>
+      </c>
+      <c r="D1261" t="s">
+        <v>3761</v>
+      </c>
+      <c r="E1261" t="s">
+        <v>3762</v>
+      </c>
+      <c r="F1261" t="s">
+        <v>3763</v>
+      </c>
+      <c r="G1261" t="s">
+        <v>417</v>
+      </c>
+      <c r="H1261">
+        <v>0</v>
+      </c>
+      <c r="I1261" t="s">
+        <v>3764</v>
+      </c>
+      <c r="J1261"/>
+      <c r="K1261"/>
+      <c r="L1261"/>
+      <c r="M1261"/>
+      <c r="N1261">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>